<commit_message>
Add check params in services, and some?
</commit_message>
<xml_diff>
--- a/backend/src/lib/excel-templates/vehicle/tripTicketTemplate.xlsx
+++ b/backend/src/lib/excel-templates/vehicle/tripTicketTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\SYSTEM EXCEL FILES\Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{636EA081-5ECC-494B-B931-B4A4D3175A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46F240B6-0CCC-476A-A2C4-041A20A5AB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -436,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -504,6 +504,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -513,6 +514,12 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -528,9 +535,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="20" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -549,6 +553,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -575,27 +582,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="6"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <border>
         <bottom style="thin">
@@ -1173,70 +1165,70 @@
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
       <c r="L2" s="13"/>
       <c r="M2" s="13"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-      <c r="J3" s="29"/>
-      <c r="K3" s="29"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
       <c r="L3" s="13"/>
       <c r="M3" s="13"/>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
     </row>
@@ -1244,99 +1236,99 @@
       <c r="B7" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="53"/>
-      <c r="D7" s="54"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="34"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1">
       <c r="C8" s="28"/>
-      <c r="J8" s="32" t="s">
+      <c r="J8" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="32"/>
+      <c r="K8" s="35"/>
     </row>
     <row r="9" spans="1:13">
       <c r="K9" s="4"/>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
     </row>
     <row r="13" spans="1:13">
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="36"/>
-      <c r="J13" s="36"/>
-      <c r="K13" s="36"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
     </row>
     <row r="14" spans="1:13">
       <c r="B14" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
+      <c r="H14" s="39"/>
+      <c r="I14" s="39"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
     </row>
     <row r="15" spans="1:13" ht="21" customHeight="1">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
       <c r="G15" s="5"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="36"/>
-      <c r="J15" s="36"/>
-      <c r="K15" s="36"/>
+      <c r="H15" s="39"/>
+      <c r="I15" s="39"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="39"/>
     </row>
     <row r="16" spans="1:13" ht="21" customHeight="1">
       <c r="B16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="36"/>
-      <c r="I16" s="36"/>
-      <c r="J16" s="36"/>
-      <c r="K16" s="36"/>
+      <c r="H16" s="39"/>
+      <c r="I16" s="39"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
     </row>
     <row r="17" spans="1:12" ht="11.25" customHeight="1">
       <c r="H17" s="5"/>
@@ -1349,26 +1341,26 @@
         <v>47</v>
       </c>
       <c r="C18" s="5"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="35"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="38"/>
+      <c r="K18" s="38"/>
+      <c r="L18" s="38"/>
     </row>
     <row r="19" spans="1:12">
-      <c r="D19" s="37"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
-      <c r="J19" s="35"/>
-      <c r="K19" s="35"/>
-      <c r="L19" s="35"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="46"/>
+      <c r="I19" s="46"/>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="L19" s="29"/>
     </row>
     <row r="20" spans="1:12">
       <c r="D20" s="5"/>
@@ -1382,31 +1374,31 @@
       <c r="L20" s="5"/>
     </row>
     <row r="21" spans="1:12">
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
+      <c r="J21" s="38"/>
+      <c r="K21" s="38"/>
+      <c r="L21" s="38"/>
     </row>
     <row r="23" spans="1:12">
-      <c r="A23" s="35" t="s">
+      <c r="A23" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
-      <c r="K23" s="35"/>
-      <c r="L23" s="35"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="38"/>
+      <c r="J23" s="38"/>
+      <c r="K23" s="38"/>
+      <c r="L23" s="38"/>
     </row>
     <row r="24" spans="1:12" ht="15" customHeight="1">
       <c r="A24" s="5"/>
@@ -1438,17 +1430,17 @@
     </row>
     <row r="26" spans="1:12" ht="15" customHeight="1">
       <c r="A26" s="5"/>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="44" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="43" t="s">
+      <c r="C26" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="43"/>
-      <c r="E26" s="42" t="s">
+      <c r="D26" s="45"/>
+      <c r="E26" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="F26" s="42"/>
+      <c r="F26" s="44"/>
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -1458,11 +1450,11 @@
     </row>
     <row r="27" spans="1:12" ht="15" customHeight="1">
       <c r="A27" s="5"/>
-      <c r="B27" s="42"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="42"/>
-      <c r="F27" s="42"/>
+      <c r="B27" s="44"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
@@ -1473,10 +1465,10 @@
     <row r="28" spans="1:12">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
-      <c r="C28" s="38"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="41"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="43"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -1487,10 +1479,10 @@
     <row r="29" spans="1:12">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="44"/>
-      <c r="F29" s="41"/>
+      <c r="C29" s="40"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="43"/>
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
@@ -1501,10 +1493,10 @@
     <row r="30" spans="1:12">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="44"/>
-      <c r="F30" s="41"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="43"/>
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
@@ -1515,10 +1507,10 @@
     <row r="31" spans="1:12">
       <c r="A31" s="5"/>
       <c r="B31" s="6"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="44"/>
-      <c r="F31" s="41"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="43"/>
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
@@ -1529,10 +1521,10 @@
     <row r="32" spans="1:12">
       <c r="A32" s="5"/>
       <c r="B32" s="7"/>
-      <c r="C32" s="39"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="44"/>
-      <c r="F32" s="41"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="43"/>
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
@@ -1543,10 +1535,10 @@
     <row r="33" spans="1:12">
       <c r="A33" s="5"/>
       <c r="B33" s="7"/>
-      <c r="C33" s="39"/>
-      <c r="D33" s="39"/>
-      <c r="E33" s="44"/>
-      <c r="F33" s="41"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="47"/>
+      <c r="F33" s="43"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
@@ -1580,15 +1572,15 @@
       <c r="K35" s="9"/>
     </row>
     <row r="36" spans="1:12" s="1" customFormat="1">
-      <c r="B36" s="45" t="s">
+      <c r="B36" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="45"/>
-      <c r="G36" s="45"/>
-      <c r="H36" s="45"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="48"/>
+      <c r="G36" s="48"/>
+      <c r="H36" s="48"/>
       <c r="I36" s="9"/>
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
@@ -1596,12 +1588,12 @@
     </row>
     <row r="37" spans="1:12" s="1" customFormat="1">
       <c r="B37" s="9"/>
-      <c r="C37" s="45" t="s">
+      <c r="C37" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="45"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="48"/>
       <c r="G37" s="9"/>
       <c r="H37" s="10"/>
       <c r="I37" s="9"/>
@@ -1613,12 +1605,12 @@
     </row>
     <row r="38" spans="1:12" s="1" customFormat="1">
       <c r="B38" s="9"/>
-      <c r="C38" s="45" t="s">
+      <c r="C38" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="45"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="45"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="48"/>
       <c r="G38" s="9"/>
       <c r="H38" s="10"/>
       <c r="I38" s="9"/>
@@ -1632,12 +1624,12 @@
     </row>
     <row r="39" spans="1:12" s="1" customFormat="1">
       <c r="B39" s="9"/>
-      <c r="C39" s="45" t="s">
+      <c r="C39" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="D39" s="45"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
+      <c r="D39" s="48"/>
+      <c r="E39" s="48"/>
+      <c r="F39" s="48"/>
       <c r="G39" s="9"/>
       <c r="H39" s="10"/>
       <c r="I39" s="9"/>
@@ -1654,9 +1646,9 @@
         <v>63</v>
       </c>
       <c r="E40" s="9"/>
-      <c r="F40" s="46"/>
-      <c r="G40" s="46"/>
-      <c r="H40" s="46"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="49"/>
+      <c r="H40" s="49"/>
       <c r="I40" s="12"/>
       <c r="J40" s="9" t="s">
         <v>59</v>
@@ -1665,15 +1657,15 @@
       <c r="L40" s="9"/>
     </row>
     <row r="41" spans="1:12" s="1" customFormat="1" ht="14.25" customHeight="1">
-      <c r="B41" s="47" t="s">
+      <c r="B41" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="47"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="46"/>
-      <c r="F41" s="46"/>
-      <c r="G41" s="46"/>
-      <c r="H41" s="46"/>
+      <c r="C41" s="50"/>
+      <c r="D41" s="49"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="49"/>
+      <c r="H41" s="49"/>
       <c r="I41" s="12"/>
       <c r="J41" s="1" t="s">
         <v>59</v>
@@ -1681,15 +1673,15 @@
       <c r="L41" s="9"/>
     </row>
     <row r="42" spans="1:12" s="1" customFormat="1" ht="14.25" customHeight="1">
-      <c r="B42" s="45" t="s">
+      <c r="B42" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
+      <c r="H42" s="49"/>
       <c r="I42" s="12"/>
       <c r="J42" s="1" t="s">
         <v>59</v>
@@ -1697,15 +1689,15 @@
       <c r="L42" s="9"/>
     </row>
     <row r="43" spans="1:12" s="1" customFormat="1" ht="14.25" customHeight="1">
-      <c r="B43" s="45" t="s">
+      <c r="B43" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="C43" s="45"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="46"/>
-      <c r="F43" s="46"/>
-      <c r="G43" s="46"/>
-      <c r="H43" s="46"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="49"/>
       <c r="I43" s="12"/>
       <c r="J43" s="1" t="s">
         <v>59</v>
@@ -1713,13 +1705,13 @@
       <c r="L43" s="9"/>
     </row>
     <row r="44" spans="1:12" s="1" customFormat="1" ht="14.25" customHeight="1">
-      <c r="B44" s="45" t="s">
+      <c r="B44" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="C44" s="45"/>
-      <c r="D44" s="45"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="45"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="48"/>
+      <c r="F44" s="48"/>
       <c r="G44" s="9"/>
       <c r="H44" s="9"/>
       <c r="I44" s="9"/>
@@ -1729,12 +1721,12 @@
     </row>
     <row r="45" spans="1:12" s="1" customFormat="1">
       <c r="B45" s="9"/>
-      <c r="C45" s="45" t="s">
+      <c r="C45" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="45"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="48"/>
       <c r="G45" s="9"/>
       <c r="H45" s="10"/>
       <c r="I45" s="9"/>
@@ -1746,12 +1738,12 @@
     </row>
     <row r="46" spans="1:12" s="1" customFormat="1">
       <c r="B46" s="9"/>
-      <c r="C46" s="45" t="s">
+      <c r="C46" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="45"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
+      <c r="F46" s="48"/>
       <c r="G46" s="9"/>
       <c r="H46" s="10"/>
       <c r="I46" s="9"/>
@@ -1763,12 +1755,12 @@
     </row>
     <row r="47" spans="1:12" s="1" customFormat="1" ht="14.25" customHeight="1">
       <c r="B47" s="9"/>
-      <c r="C47" s="45" t="s">
+      <c r="C47" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="45"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
+      <c r="F47" s="48"/>
       <c r="G47" s="9"/>
       <c r="H47" s="10"/>
       <c r="I47" s="9"/>
@@ -1792,18 +1784,18 @@
       <c r="L48" s="9"/>
     </row>
     <row r="49" spans="2:12" s="1" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B49" s="45" t="s">
+      <c r="B49" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="C49" s="45"/>
-      <c r="D49" s="48"/>
-      <c r="E49" s="48"/>
-      <c r="F49" s="48"/>
-      <c r="G49" s="48"/>
-      <c r="H49" s="48"/>
-      <c r="I49" s="48"/>
-      <c r="J49" s="48"/>
-      <c r="K49" s="48"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="51"/>
+      <c r="J49" s="51"/>
+      <c r="K49" s="51"/>
       <c r="L49" s="9"/>
     </row>
     <row r="50" spans="2:12" s="1" customFormat="1">
@@ -1820,18 +1812,18 @@
       <c r="L50" s="9"/>
     </row>
     <row r="51" spans="2:12" s="1" customFormat="1">
-      <c r="B51" s="49" t="s">
+      <c r="B51" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="C51" s="49"/>
-      <c r="D51" s="49"/>
-      <c r="E51" s="49"/>
-      <c r="F51" s="49"/>
-      <c r="G51" s="49"/>
-      <c r="H51" s="49"/>
-      <c r="I51" s="49"/>
-      <c r="J51" s="49"/>
-      <c r="K51" s="49"/>
+      <c r="C51" s="52"/>
+      <c r="D51" s="52"/>
+      <c r="E51" s="52"/>
+      <c r="F51" s="52"/>
+      <c r="G51" s="52"/>
+      <c r="H51" s="52"/>
+      <c r="I51" s="52"/>
+      <c r="J51" s="52"/>
+      <c r="K51" s="52"/>
       <c r="L51" s="9"/>
     </row>
     <row r="52" spans="2:12" s="1" customFormat="1">
@@ -1856,8 +1848,8 @@
       <c r="G53" s="9"/>
       <c r="H53" s="11"/>
       <c r="I53" s="9"/>
-      <c r="J53" s="50"/>
-      <c r="K53" s="50"/>
+      <c r="J53" s="53"/>
+      <c r="K53" s="53"/>
       <c r="L53" s="9"/>
     </row>
     <row r="54" spans="2:12" s="1" customFormat="1">
@@ -1871,8 +1863,8 @@
         <v>73</v>
       </c>
       <c r="I54" s="9"/>
-      <c r="J54" s="50"/>
-      <c r="K54" s="50"/>
+      <c r="J54" s="53"/>
+      <c r="K54" s="53"/>
       <c r="L54" s="9"/>
     </row>
     <row r="55" spans="2:12" s="1" customFormat="1">
@@ -1889,18 +1881,18 @@
       <c r="L55" s="9"/>
     </row>
     <row r="56" spans="2:12" s="1" customFormat="1">
-      <c r="B56" s="49" t="s">
+      <c r="B56" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="C56" s="49"/>
-      <c r="D56" s="49"/>
-      <c r="E56" s="49"/>
-      <c r="F56" s="49"/>
-      <c r="G56" s="49"/>
-      <c r="H56" s="49"/>
-      <c r="I56" s="49"/>
-      <c r="J56" s="49"/>
-      <c r="K56" s="49"/>
+      <c r="C56" s="52"/>
+      <c r="D56" s="52"/>
+      <c r="E56" s="52"/>
+      <c r="F56" s="52"/>
+      <c r="G56" s="52"/>
+      <c r="H56" s="52"/>
+      <c r="I56" s="52"/>
+      <c r="J56" s="52"/>
+      <c r="K56" s="52"/>
       <c r="L56" s="9"/>
     </row>
     <row r="57" spans="2:12" s="1" customFormat="1">
@@ -1917,11 +1909,11 @@
       <c r="L57" s="9"/>
     </row>
     <row r="58" spans="2:12" s="1" customFormat="1" ht="14.25" customHeight="1">
-      <c r="B58" s="50" t="s">
+      <c r="B58" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="C58" s="50"/>
-      <c r="D58" s="50"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="53"/>
       <c r="E58" s="12"/>
       <c r="F58" s="12" t="s">
         <v>75</v>
@@ -1937,9 +1929,9 @@
       <c r="L58" s="9"/>
     </row>
     <row r="59" spans="2:12" s="1" customFormat="1">
-      <c r="B59" s="48"/>
-      <c r="C59" s="48"/>
-      <c r="D59" s="48"/>
+      <c r="B59" s="51"/>
+      <c r="C59" s="51"/>
+      <c r="D59" s="51"/>
       <c r="E59" s="9"/>
       <c r="F59" s="10"/>
       <c r="G59" s="9"/>
@@ -1949,9 +1941,9 @@
       <c r="L59" s="9"/>
     </row>
     <row r="60" spans="2:12" s="1" customFormat="1">
-      <c r="B60" s="48"/>
-      <c r="C60" s="48"/>
-      <c r="D60" s="48"/>
+      <c r="B60" s="51"/>
+      <c r="C60" s="51"/>
+      <c r="D60" s="51"/>
       <c r="E60" s="9"/>
       <c r="F60" s="10"/>
       <c r="G60" s="9"/>
@@ -1962,9 +1954,9 @@
       <c r="L60" s="9"/>
     </row>
     <row r="61" spans="2:12" s="1" customFormat="1">
-      <c r="B61" s="48"/>
-      <c r="C61" s="48"/>
-      <c r="D61" s="48"/>
+      <c r="B61" s="51"/>
+      <c r="C61" s="51"/>
+      <c r="D61" s="51"/>
       <c r="E61" s="9"/>
       <c r="F61" s="10"/>
       <c r="G61" s="9"/>
@@ -1975,9 +1967,9 @@
       <c r="L61" s="9"/>
     </row>
     <row r="62" spans="2:12" s="1" customFormat="1">
-      <c r="B62" s="48"/>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="B62" s="51"/>
+      <c r="C62" s="51"/>
+      <c r="D62" s="51"/>
       <c r="E62" s="9"/>
       <c r="F62" s="10"/>
       <c r="G62" s="9"/>
@@ -1988,9 +1980,9 @@
       <c r="L62" s="9"/>
     </row>
     <row r="63" spans="2:12" s="1" customFormat="1">
-      <c r="B63" s="48"/>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
+      <c r="B63" s="51"/>
+      <c r="C63" s="51"/>
+      <c r="D63" s="51"/>
       <c r="E63" s="9"/>
       <c r="F63" s="10"/>
       <c r="G63" s="9"/>
@@ -2022,44 +2014,44 @@
       </c>
     </row>
     <row r="68" spans="2:12">
-      <c r="B68" s="51"/>
-      <c r="C68" s="51"/>
-      <c r="D68" s="51"/>
-      <c r="E68" s="51"/>
-      <c r="F68" s="51"/>
+      <c r="B68" s="54"/>
+      <c r="C68" s="54"/>
+      <c r="D68" s="54"/>
+      <c r="E68" s="54"/>
+      <c r="F68" s="54"/>
       <c r="G68" s="14"/>
       <c r="H68" s="15"/>
       <c r="J68" s="15"/>
       <c r="K68" s="15"/>
     </row>
     <row r="69" spans="2:12">
-      <c r="B69" s="34" t="s">
+      <c r="B69" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="C69" s="34"/>
-      <c r="D69" s="34"/>
-      <c r="E69" s="34"/>
-      <c r="F69" s="34"/>
+      <c r="C69" s="37"/>
+      <c r="D69" s="37"/>
+      <c r="E69" s="37"/>
+      <c r="F69" s="37"/>
       <c r="G69" s="4"/>
       <c r="H69" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="J69" s="52"/>
-      <c r="K69" s="52"/>
+      <c r="J69" s="55"/>
+      <c r="K69" s="55"/>
     </row>
     <row r="70" spans="2:12">
-      <c r="J70" s="35"/>
-      <c r="K70" s="35"/>
-      <c r="L70" s="35"/>
+      <c r="J70" s="38"/>
+      <c r="K70" s="38"/>
+      <c r="L70" s="38"/>
     </row>
     <row r="88" spans="6:11">
       <c r="H88" s="17"/>
       <c r="I88" s="17"/>
     </row>
     <row r="91" spans="6:11">
-      <c r="F91" s="34"/>
-      <c r="G91" s="34"/>
-      <c r="H91" s="34"/>
+      <c r="F91" s="37"/>
+      <c r="G91" s="37"/>
+      <c r="H91" s="37"/>
       <c r="I91" s="4"/>
       <c r="K91" s="4"/>
     </row>
@@ -2083,34 +2075,34 @@
     <mergeCell ref="J54:K54"/>
     <mergeCell ref="B56:K56"/>
     <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B44:F44"/>
     <mergeCell ref="C45:F45"/>
     <mergeCell ref="C46:F46"/>
     <mergeCell ref="C47:F47"/>
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="D49:K49"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="D41:H41"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="D42:H42"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="D43:H43"/>
-    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B36:H36"/>
     <mergeCell ref="C37:F37"/>
     <mergeCell ref="C38:F38"/>
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="F40:H40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="E33:F33"/>
-    <mergeCell ref="B36:H36"/>
+    <mergeCell ref="D19:K19"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="D19:L19"/>
     <mergeCell ref="D21:L21"/>
     <mergeCell ref="A23:L23"/>
     <mergeCell ref="C28:D28"/>
@@ -2136,7 +2128,7 @@
     <mergeCell ref="C7:D7"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:D7">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$C$7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>